<commit_message>
chore(arena): update challenger models to latest versions
- Replace Kimi K2.5/Minimax M2.5/Qwen 3.5 with DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6 across arenas
- Add new challenger for arena 7 (智能文档翻译系统)
- Update CSV, XLSX, and both JSON language files

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code +Kimi K2.5/Minimax M2.5/Qwen 3.5 + Metaso</t>
+          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -579,7 +579,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>云端版：Lovable + GLM-5/Minimax M2.5/Qwen 3.5 + Claude Code</t>
+          <t>云端版：Lovable + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6/Minimax M2.7 + Claude Code</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + Kimi K2.5/Minimax M2.5/Qwen 3.5  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N4"/>
@@ -745,7 +745,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>私部署版：OpenClaw + Claude Opus 4.6  + FFmpeg + Qwen3-ASR + Qwen3-TTS</t>
+          <t>私部署版：OpenClaw + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6  + FFmpeg + Qwen3-ASR + Qwen3-TTS</t>
         </is>
       </c>
       <c r="N5"/>
@@ -817,7 +817,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t xml:space="preserve">私部署版：BISHENG + Kimi K2.5/Minimax M2.5/Qwen 3.5 </t>
+          <t>私部署版：BISHENG + DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6/Minimax M2.7</t>
         </is>
       </c>
       <c r="N6"/>
@@ -962,7 +962,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>寻找攻擂者</t>
+          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6</t>
         </is>
       </c>
       <c r="N8"/>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t xml:space="preserve">私部署版：Coze + Kimi K2.5/Minimax M2.5/Qwen 3.5 </t>
+          <t>私部署版：Coze +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6</t>
         </is>
       </c>
       <c r="N12"/>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N13"/>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>私部署版：LangChain + Kimi K2.5/Minimax M2.5/Qwen 3.5  + Pydantic + unstructured + Faiss</t>
+          <t>私部署版：LangChain +  DeepSeek V4 Pro/GLM 5.1/Kimi K2.6/Minimax M2.7/Qwen 3.6  + Pydantic + unstructured + Faiss</t>
         </is>
       </c>
       <c r="N14"/>

</xml_diff>

<commit_message>
chore(arena): update arena 1 champion to DeepSeek V4 Pro + StepSearch
- Change arena 1 champion from GLM 5 + Metaso to DeepSeek V4 Pro + StepSearch
- Update benchmark scores (51.86→53.54) and rankings
- Add StepSearch MCP configuration to tech-configuration
- Remove "最近审阅"/"Last Reviewed" date fields across all arenas
- Refresh update dates to 2026-05-18 across all arenas

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -442,14 +442,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + GLM 5 + Metaso</t>
+          <t>私部署版：Claude Code + DeepSeek V4 Pro + StepSearch</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Claude Code (by Anthropic) GitHub：https://github.com/anthropics/claude-code
-Metaso MCP (by 秘塔科技) 文档：https://www.modelscope.cn/mcp/servers/metasota/metaso-search
-GLM-5(by 智谱) GitHub：https://github.com/zai-org/GLM-5</t>
+StepSearch MCP (by 阶跃星辰) 文档：https://platform.stepfun.com/docs/zh/step-plan/integrations/search-mcp
+DeepSeek-V4-Pro(by 深度求索) Hugging Face：https://huggingface.co/deepseek-ai/DeepSeek-V4-Pro</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
+          <t>私部署版：Hermes Agent + MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>